<commit_message>
case2-green-methanol: lamuzhuoga group03 第九讲作业提交
</commit_message>
<xml_diff>
--- a/groups/group-03/lecture9-20261022-classroom_case1/code_implementation/case1_calculation_results.xlsx
+++ b/groups/group-03/lecture9-20261022-classroom_case1/code_implementation/case1_calculation_results.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_MFA_物质平衡" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_LCA_碳足迹" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_TEA_生产成本" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_收率敏感度" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_关键结论汇总" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="1_MFA_物质平衡" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2_LCA_碳足迹" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="3_TEA_生产成本" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4_收率敏感度" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="5_关键结论汇总" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -647,13 +647,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>636</v>
+        <v>636.0000000000001</v>
       </c>
       <c r="C9" t="n">
         <v>194</v>
       </c>
       <c r="D9" t="n">
-        <v>-442</v>
+        <v>-442.0000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>